<commit_message>
ajustes nos arquivos de importação
</commit_message>
<xml_diff>
--- a/Backups/modelo_importacao_contas(1).xlsx
+++ b/Backups/modelo_importacao_contas(1).xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djjun\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pessoal\ArquitetoDeValor\Backups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC9A4CB4-519E-4AF4-BE55-8A9D15DA2772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0572DC2-F295-4349-A764-E9E060A46195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Contas" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Contas!$A$1:$E$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Contas!$A$1:$E$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="40">
   <si>
     <t>nome</t>
   </si>
@@ -119,27 +119,18 @@
     <t>Cartão Inter</t>
   </si>
   <si>
-    <t>Inv pagpank</t>
-  </si>
-  <si>
     <t>Cartão PicPay</t>
   </si>
   <si>
     <t>Banco 99</t>
   </si>
   <si>
-    <t>Inv Null</t>
-  </si>
-  <si>
     <t>Banco C6</t>
   </si>
   <si>
     <t>Cartão C6</t>
   </si>
   <si>
-    <t>Inv c6</t>
-  </si>
-  <si>
     <t>Inv. Null</t>
   </si>
   <si>
@@ -155,9 +146,6 @@
     <t>Inv. Inter US</t>
   </si>
   <si>
-    <t>Inv Merc. Pago</t>
-  </si>
-  <si>
     <t>Banco Astropay</t>
   </si>
   <si>
@@ -165,6 +153,9 @@
   </si>
   <si>
     <t>CARTAO</t>
+  </si>
+  <si>
+    <t>Inv. Merc. Pago</t>
   </si>
 </sst>
 </file>
@@ -229,7 +220,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -246,13 +237,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -595,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.875" style="7" customWidth="1"/>
@@ -620,10 +608,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -634,7 +622,7 @@
         <v>21</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -645,7 +633,7 @@
         <v>26</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -656,7 +644,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -664,10 +652,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -678,7 +666,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -686,10 +674,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -700,7 +688,7 @@
         <v>18</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -711,7 +699,7 @@
         <v>14</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -722,7 +710,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -741,7 +729,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>4</v>
@@ -752,7 +740,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>4</v>
@@ -763,7 +751,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>4</v>
@@ -851,7 +839,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>5</v>
@@ -861,8 +849,8 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>33</v>
+      <c r="A24" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>5</v>
@@ -872,8 +860,8 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>39</v>
+      <c r="A25" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>5</v>
@@ -883,10 +871,10 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="3" t="s">
+      <c r="A26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C26">
@@ -895,9 +883,9 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C27">
@@ -906,7 +894,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>5</v>
@@ -917,7 +905,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>5</v>
@@ -928,7 +916,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>5</v>
@@ -938,8 +926,8 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>24</v>
+      <c r="A31" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>5</v>
@@ -950,7 +938,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>5</v>
@@ -961,7 +949,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>5</v>
@@ -972,7 +960,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>5</v>
@@ -981,43 +969,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D37">
-    <sortCondition ref="B2:B37"/>
+  <autoFilter ref="A1:E34" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D34">
+    <sortCondition ref="B2:B34"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>

</xml_diff>